<commit_message>
Fix acceptance history and exception coverage
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample-data/import_history/02_gl_batch_039.xlsx
+++ b/sample-data/import_history/02_gl_batch_039.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GL_Actuals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ControlTotals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GL_Actuals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ControlTotals" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6903,14 +6903,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>net</t>
+          <t>debit</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>18400000</v>
       </c>
       <c r="D2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix acceptance history and exception coverage (#3)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample-data/import_history/02_gl_batch_039.xlsx
+++ b/sample-data/import_history/02_gl_batch_039.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GL_Actuals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ControlTotals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GL_Actuals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ControlTotals" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6903,14 +6903,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>net</t>
+          <t>debit</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>18400000</v>
       </c>
       <c r="D2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>